<commit_message>
Reorganize character images and add 9 characters with 5 new skills
- Move character art into images/chars/game_characters_transparent_1/
  (full body) and game_characters_faces/ (marker face crops), updating
  charImageSrc()/charFaceSrc() and adding per-character filename
  overrides where the asset name doesn't match the internal charId
  (trapper, ogre, and the 9 new characters).
- Rebalance guardian/lancer/archer/sniper and rename ogre's display
  name to Berserker per UC's updated AFBElist.xlsx.
- Add 9 new characters (poisoner, gatekeeper, ashigaru, medic,
  lonewolf, hunter, bard, scout, king) and implement their 5 new
  skills (territory, single-target heal, lone wolf, march, blood
  scent) in the battle simulator.
- Update the design doc and CLAUDE.md to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AFBElist.xlsx
+++ b/AFBElist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\遊ぶところ\ゲーム制作\Auto_Formation_Battle_Encounter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E2EE9F-AA56-4C27-9DC4-7A27CF0F8478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81119CEE-46FC-41C8-A3FE-C8645215772D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1B17E940-1388-48E2-89F6-95B4CC23EF03}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="166">
   <si>
     <t>スキル名称</t>
     <rPh sb="3" eb="5">
@@ -295,22 +295,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>５行動力消費するたびにこのキャラの攻撃範囲にいる味方キャラはHPを20回復する</t>
-    <rPh sb="1" eb="6">
-      <t>コウドウリョクショウヒ</t>
-    </rPh>
-    <rPh sb="17" eb="21">
-      <t>コウゲキハンイ</t>
-    </rPh>
-    <rPh sb="24" eb="26">
-      <t>ミカタ</t>
-    </rPh>
-    <rPh sb="35" eb="37">
-      <t>カイフク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>毒</t>
     <rPh sb="0" eb="1">
       <t>ドク</t>
@@ -511,9 +495,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>名前(仮)</t>
-  </si>
-  <si>
     <t>値段</t>
   </si>
   <si>
@@ -550,15 +531,9 @@
     <t>陣形の核。隣に並べて真価</t>
   </si>
   <si>
-    <t>射程ボーナス2、攻撃消費2</t>
-  </si>
-  <si>
     <t>全方位射程3の遠隔</t>
   </si>
   <si>
-    <t>射撃5、攻撃消費3</t>
-  </si>
-  <si>
     <t>罠設置</t>
   </si>
   <si>
@@ -596,13 +571,7 @@
     <t>スナイパー</t>
   </si>
   <si>
-    <t>トラッパー</t>
-  </si>
-  <si>
     <t>クレリック</t>
-  </si>
-  <si>
-    <t>オーガ</t>
   </si>
   <si>
     <t>猫</t>
@@ -645,6 +614,451 @@
     <t>鹿</t>
     <rPh sb="0" eb="1">
       <t>シカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>蜘蛛　</t>
+    <rPh sb="0" eb="2">
+      <t>クモ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>トラッパー</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>毒使い</t>
+    <rPh sb="0" eb="2">
+      <t>ドクツカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>バーサーカー</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>役職</t>
+    <rPh sb="0" eb="2">
+      <t>ヤクショク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>孤高</t>
+    <rPh sb="0" eb="2">
+      <t>ココウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ドーベルマン</t>
+  </si>
+  <si>
+    <t>門番</t>
+  </si>
+  <si>
+    <t>柴犬</t>
+  </si>
+  <si>
+    <t>侍</t>
+  </si>
+  <si>
+    <t>ビーバー</t>
+  </si>
+  <si>
+    <t>クラフター</t>
+  </si>
+  <si>
+    <t>ライオン</t>
+  </si>
+  <si>
+    <t>王者</t>
+  </si>
+  <si>
+    <t>トラ</t>
+  </si>
+  <si>
+    <t>狩人</t>
+  </si>
+  <si>
+    <t>弱った獲物を高速で狩り切る</t>
+  </si>
+  <si>
+    <t>ヒョウ</t>
+  </si>
+  <si>
+    <t>フェンサー</t>
+  </si>
+  <si>
+    <t>ヒットアンドアウェイ</t>
+  </si>
+  <si>
+    <t>殴って離脱。近接に捕まらない剣士</t>
+  </si>
+  <si>
+    <t>オオカミ</t>
+  </si>
+  <si>
+    <t>孤高</t>
+  </si>
+  <si>
+    <t>連携ゲーの逆張り。単独行動で強化</t>
+  </si>
+  <si>
+    <t>キリン</t>
+  </si>
+  <si>
+    <t>僧侶</t>
+  </si>
+  <si>
+    <t>聖域、射程ボーナス1</t>
+  </si>
+  <si>
+    <t>半径2の回復＋毒解除。首が長い＝範囲広い</t>
+  </si>
+  <si>
+    <t>ウマ</t>
+  </si>
+  <si>
+    <t>キャリアー</t>
+  </si>
+  <si>
+    <t>牽引</t>
+  </si>
+  <si>
+    <t>味方を連れて走る機動展開の要</t>
+  </si>
+  <si>
+    <t>リス</t>
+  </si>
+  <si>
+    <t>足軽</t>
+  </si>
+  <si>
+    <t>最安値。数で壁を作る／連携の起点</t>
+  </si>
+  <si>
+    <t>レッサーパンダ</t>
+  </si>
+  <si>
+    <t>学者</t>
+  </si>
+  <si>
+    <t>解析、射程ボーナス1</t>
+  </si>
+  <si>
+    <t>敵の防御を崩すデバフオーラ</t>
+  </si>
+  <si>
+    <t>ウシ</t>
+  </si>
+  <si>
+    <t>衛生兵</t>
+  </si>
+  <si>
+    <t>治療</t>
+  </si>
+  <si>
+    <t>単体大回復。フクロウと役割分担</t>
+  </si>
+  <si>
+    <t>サル</t>
+  </si>
+  <si>
+    <t>マーチャント</t>
+  </si>
+  <si>
+    <t>商売</t>
+  </si>
+  <si>
+    <t>生存＝金策。守り切る経済ユニット</t>
+  </si>
+  <si>
+    <t>カンガルー</t>
+  </si>
+  <si>
+    <t>ボクサー</t>
+  </si>
+  <si>
+    <t>ワンツー</t>
+  </si>
+  <si>
+    <t>1回の攻撃行動で2発。手数の格闘家</t>
+  </si>
+  <si>
+    <t>タヌキ</t>
+  </si>
+  <si>
+    <t>忍者</t>
+  </si>
+  <si>
+    <t>変化、身軽</t>
+  </si>
+  <si>
+    <t>正体を偽る。秘匿配置ルールと相性抜群</t>
+  </si>
+  <si>
+    <t>ゾウ</t>
+  </si>
+  <si>
+    <t>タンク</t>
+  </si>
+  <si>
+    <t>巨体</t>
+  </si>
+  <si>
+    <t>最大HP。押し込み・引き寄せ無効の動く城壁</t>
+  </si>
+  <si>
+    <t>フェネック</t>
+  </si>
+  <si>
+    <t>吟遊詩人</t>
+  </si>
+  <si>
+    <t>味方の行動力を増やす応援団</t>
+  </si>
+  <si>
+    <t>ヤマアラシ</t>
+  </si>
+  <si>
+    <t>オウム</t>
+  </si>
+  <si>
+    <t>バード</t>
+  </si>
+  <si>
+    <t>物真似</t>
+  </si>
+  <si>
+    <t>味方のスキルをコピーする万能枠</t>
+  </si>
+  <si>
+    <t>サイ</t>
+  </si>
+  <si>
+    <t>グラディエーター</t>
+  </si>
+  <si>
+    <t>突進</t>
+  </si>
+  <si>
+    <t>助走をつけて轢く重戦車</t>
+  </si>
+  <si>
+    <t>カラス</t>
+  </si>
+  <si>
+    <t>クリーナー</t>
+  </si>
+  <si>
+    <t>死肉あさり</t>
+  </si>
+  <si>
+    <t>死体が出るほど元気になる戦場の掃除屋</t>
+  </si>
+  <si>
+    <t>縄張り</t>
+    <rPh sb="0" eb="2">
+      <t>ナワバ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自陣最強番犬</t>
+    <rPh sb="0" eb="4">
+      <t>ジジンサイキョウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自陣エリアにいる間攻撃力が２倍になる</t>
+    <rPh sb="0" eb="2">
+      <t>ジジン</t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t>アイダ</t>
+    </rPh>
+    <rPh sb="9" eb="12">
+      <t>コウゲキリョク</t>
+    </rPh>
+    <rPh sb="14" eb="15">
+      <t>バイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>単体回復N</t>
+    <rPh sb="0" eb="4">
+      <t>タンタイカイフク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>3行動力消費するたびにこのキャラの攻撃範囲にいる味方キャラはHPを20回復する</t>
+    <rPh sb="1" eb="6">
+      <t>コウドウリョクショウヒ</t>
+    </rPh>
+    <rPh sb="17" eb="21">
+      <t>コウゲキハンイ</t>
+    </rPh>
+    <rPh sb="24" eb="26">
+      <t>ミカタ</t>
+    </rPh>
+    <rPh sb="35" eb="37">
+      <t>カイフク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>このキャラの攻撃範囲にいる味方キャラはHPを20回復する(行動力１消費。攻撃よりも優先される)</t>
+    <rPh sb="6" eb="10">
+      <t>コウゲキハンイ</t>
+    </rPh>
+    <rPh sb="29" eb="32">
+      <t>コウドウリョク</t>
+    </rPh>
+    <rPh sb="33" eb="35">
+      <t>ショウヒ</t>
+    </rPh>
+    <rPh sb="36" eb="38">
+      <t>コウゲキ</t>
+    </rPh>
+    <rPh sb="41" eb="43">
+      <t>ユウセン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自分の3マス以内に味方がいない時、攻撃力+20</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>行進曲</t>
+    <rPh sb="0" eb="3">
+      <t>コウシンキョク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>このキャラ自身が行動力を3消費するたび、攻撃範囲内の味方（自分を除く）の行動力+1(１ラウンドに付き5回まで)</t>
+    <rPh sb="48" eb="49">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="51" eb="52">
+      <t>カイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>一匹狼</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>指示は聞かず最も近い相手キャラに最短で近づく</t>
+    <rPh sb="0" eb="2">
+      <t>シジ</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="6" eb="7">
+      <t>モット</t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t>チカ</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>アイテ</t>
+    </rPh>
+    <rPh sb="16" eb="18">
+      <t>サイタン</t>
+    </rPh>
+    <rPh sb="19" eb="20">
+      <t>チカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>移動ボーナス1、血の匂い</t>
+    <rPh sb="8" eb="9">
+      <t>チ</t>
+    </rPh>
+    <rPh sb="10" eb="11">
+      <t>ニオ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>血の匂い</t>
+    <rPh sb="0" eb="1">
+      <t>チ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ニオ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>まだ検討中</t>
+    <rPh sb="2" eb="5">
+      <t>ケントウチュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>採用</t>
+    <rPh sb="0" eb="2">
+      <t>サイヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>スカウト</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>行進曲、射程ボーナス1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>遠距離連携攻撃、射程ボーナス1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>味方の攻撃に合わせる支援役</t>
+    <rPh sb="3" eb="5">
+      <t>コウゲキ</t>
+    </rPh>
+    <rPh sb="6" eb="7">
+      <t>ア</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>シエン</t>
+    </rPh>
+    <rPh sb="12" eb="13">
+      <t>ヤク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>射程ボーナス2、攻撃消費1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>射撃8、攻撃消費2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>天下無双まさに王者</t>
+    <rPh sb="0" eb="4">
+      <t>テンカムソウ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>オウジャ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -653,7 +1067,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -678,6 +1092,19 @@
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="游ゴシック"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Meiryo"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -687,7 +1114,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -710,13 +1137,29 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -738,9 +1181,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
+    <cellStyle name="標準 2" xfId="1" xr:uid="{233F4D1B-A9BE-47CB-94E5-FDAD402B227E}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1052,24 +1508,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19769DCE-A1D1-47E3-BFED-8EA4734B55A4}">
-  <dimension ref="B2:D19"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <dimension ref="B2:D30"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="9" style="4"/>
     <col min="3" max="3" width="24.25" customWidth="1"/>
-    <col min="4" max="4" width="53.875" customWidth="1"/>
+    <col min="4" max="4" width="53.875" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:4">
       <c r="B2" s="3"/>
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:4" ht="36.75" customHeight="1">
       <c r="B3" s="3">
         <v>1</v>
       </c>
@@ -1080,7 +1536,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="56.25" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:4" ht="56.25">
       <c r="B4" s="3">
         <v>2</v>
       </c>
@@ -1091,7 +1547,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="56.25" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:4" ht="56.25">
       <c r="B5" s="3">
         <v>3</v>
       </c>
@@ -1102,18 +1558,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:4">
       <c r="B6" s="3">
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:4">
       <c r="B7" s="3">
         <v>5</v>
       </c>
@@ -1124,7 +1580,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="37.5" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:4" ht="37.5">
       <c r="B8" s="3">
         <v>6</v>
       </c>
@@ -1135,7 +1591,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="37.5" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:4" ht="37.5">
       <c r="B9" s="3">
         <v>7</v>
       </c>
@@ -1146,7 +1602,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="37.5" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:4" ht="37.5">
       <c r="B10" s="3">
         <v>8</v>
       </c>
@@ -1157,7 +1613,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="37.5" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:4" ht="37.5">
       <c r="B11" s="3">
         <v>9</v>
       </c>
@@ -1165,21 +1621,21 @@
         <v>19</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4" ht="37.5" x14ac:dyDescent="0.4">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" ht="37.5">
       <c r="B12" s="3">
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.4">
+    </row>
+    <row r="13" spans="2:4">
       <c r="B13" s="3">
         <v>11</v>
       </c>
@@ -1190,71 +1646,168 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:4">
       <c r="B14" s="3">
         <v>12</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" ht="37.5" x14ac:dyDescent="0.4">
+    </row>
+    <row r="15" spans="2:4" ht="37.5">
       <c r="B15" s="3">
         <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" ht="56.25" x14ac:dyDescent="0.4">
+    </row>
+    <row r="16" spans="2:4" ht="56.25">
       <c r="B16" s="3">
         <v>14</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.4">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4">
       <c r="B17" s="3">
         <v>15</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.4">
+    </row>
+    <row r="18" spans="2:4">
       <c r="B18" s="3">
         <v>16</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.4">
+    </row>
+    <row r="19" spans="2:4">
       <c r="B19" s="3">
         <v>17</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>34</v>
-      </c>
+    </row>
+    <row r="20" spans="2:4">
+      <c r="B20" s="3">
+        <v>18</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" ht="37.5">
+      <c r="B21" s="3">
+        <v>19</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4">
+      <c r="B22" s="3">
+        <v>20</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" ht="37.5">
+      <c r="B23" s="3">
+        <v>21</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4">
+      <c r="B24" s="3">
+        <v>22</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4">
+      <c r="B25" s="3">
+        <v>23</v>
+      </c>
+      <c r="C25" s="1"/>
+      <c r="D25" s="2"/>
+    </row>
+    <row r="26" spans="2:4">
+      <c r="B26" s="3">
+        <v>24</v>
+      </c>
+      <c r="C26" s="1"/>
+      <c r="D26" s="2"/>
+    </row>
+    <row r="27" spans="2:4">
+      <c r="B27" s="3">
+        <v>25</v>
+      </c>
+      <c r="C27" s="1"/>
+      <c r="D27" s="2"/>
+    </row>
+    <row r="28" spans="2:4">
+      <c r="B28" s="3">
+        <v>26</v>
+      </c>
+      <c r="C28" s="1"/>
+      <c r="D28" s="2"/>
+    </row>
+    <row r="29" spans="2:4">
+      <c r="B29" s="3">
+        <v>27</v>
+      </c>
+      <c r="C29" s="1"/>
+      <c r="D29" s="2"/>
+    </row>
+    <row r="30" spans="2:4">
+      <c r="B30" s="3">
+        <v>28</v>
+      </c>
+      <c r="C30" s="1"/>
+      <c r="D30" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -1264,55 +1817,92 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14515E83-A93E-48F7-8531-5F98695B0245}">
-  <dimension ref="B2:I10"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:I34"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="3" max="3" width="14.5" customWidth="1"/>
+    <col min="2" max="2" width="16.125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="14.5" style="8" customWidth="1"/>
+    <col min="4" max="7" width="9" style="8"/>
     <col min="8" max="8" width="30.625" customWidth="1"/>
     <col min="9" max="9" width="45.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="C2" s="5" t="s">
+    <row r="1" spans="1:9">
+      <c r="B1" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F1" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="G1" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="H2" s="5" t="s">
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="6">
+        <v>50</v>
+      </c>
+      <c r="E2" s="6">
+        <v>100</v>
+      </c>
+      <c r="F2" s="6">
+        <v>20</v>
+      </c>
+      <c r="G2" s="6">
+        <v>15</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C3" t="s">
-        <v>59</v>
+    <row r="3" spans="1:9">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>56</v>
       </c>
       <c r="D3" s="6">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E3" s="6">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F3" s="6">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G3" s="6">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>43</v>
@@ -1321,24 +1911,27 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" t="s">
-        <v>60</v>
+    <row r="4" spans="1:9">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>57</v>
       </c>
       <c r="D4" s="6">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E4" s="6">
-        <v>200</v>
+        <v>90</v>
       </c>
       <c r="F4" s="6">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G4" s="6">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>45</v>
@@ -1347,160 +1940,811 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" t="s">
-        <v>61</v>
+    <row r="5" spans="1:9">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="D5" s="6">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E5" s="6">
+        <v>60</v>
+      </c>
+      <c r="F5" s="6">
+        <v>25</v>
+      </c>
+      <c r="G5" s="6">
+        <v>12</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="6">
+        <v>70</v>
+      </c>
+      <c r="E6" s="6">
+        <v>50</v>
+      </c>
+      <c r="F6" s="6">
+        <v>40</v>
+      </c>
+      <c r="G6" s="6">
+        <v>10</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" s="6">
+        <v>55</v>
+      </c>
+      <c r="E7" s="6">
         <v>90</v>
       </c>
-      <c r="F5" s="6">
-        <v>20</v>
-      </c>
-      <c r="G5" s="6">
-        <v>18</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B6" t="s">
-        <v>71</v>
-      </c>
-      <c r="C6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D6" s="6">
-        <v>60</v>
-      </c>
-      <c r="E6" s="6">
-        <v>60</v>
-      </c>
-      <c r="F6" s="6">
-        <v>25</v>
-      </c>
-      <c r="G6" s="6">
-        <v>12</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B7" t="s">
-        <v>70</v>
-      </c>
-      <c r="C7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D7" s="6">
-        <v>70</v>
-      </c>
-      <c r="E7" s="6">
-        <v>50</v>
-      </c>
       <c r="F7" s="6">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G7" s="6">
         <v>10</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C8" t="s">
-        <v>64</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>60</v>
       </c>
       <c r="D8" s="6">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E8" s="6">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F8" s="6">
         <v>10</v>
       </c>
       <c r="G8" s="6">
+        <v>15</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D9" s="6">
+        <v>90</v>
+      </c>
+      <c r="E9" s="6">
+        <v>100</v>
+      </c>
+      <c r="F9" s="6">
+        <v>15</v>
+      </c>
+      <c r="G9" s="6">
+        <v>14</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="6">
+        <v>55</v>
+      </c>
+      <c r="E10" s="6">
+        <v>70</v>
+      </c>
+      <c r="F10" s="6">
+        <v>10</v>
+      </c>
+      <c r="G10" s="6">
         <v>6</v>
       </c>
-      <c r="H8" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B9" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="H10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="10">
         <v>65</v>
       </c>
-      <c r="D9" s="6">
+      <c r="E11" s="10">
+        <v>150</v>
+      </c>
+      <c r="F11" s="10">
+        <v>15</v>
+      </c>
+      <c r="G11" s="10">
+        <v>13</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="D12" s="10">
+        <v>30</v>
+      </c>
+      <c r="E12" s="10">
+        <v>50</v>
+      </c>
+      <c r="F12" s="10">
+        <v>10</v>
+      </c>
+      <c r="G12" s="10">
+        <v>14</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D13" s="10">
+        <v>75</v>
+      </c>
+      <c r="E13" s="10">
+        <v>150</v>
+      </c>
+      <c r="F13" s="10">
+        <v>5</v>
+      </c>
+      <c r="G13" s="10">
+        <v>10</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="D14" s="10">
+        <v>65</v>
+      </c>
+      <c r="E14" s="10">
+        <v>130</v>
+      </c>
+      <c r="F14" s="10">
+        <v>20</v>
+      </c>
+      <c r="G14" s="10">
+        <v>15</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="10">
+        <v>75</v>
+      </c>
+      <c r="E15" s="10">
+        <v>90</v>
+      </c>
+      <c r="F15" s="10">
+        <v>25</v>
+      </c>
+      <c r="G15" s="10">
+        <v>14</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="D16" s="10">
+        <v>80</v>
+      </c>
+      <c r="E16" s="10">
         <v>70</v>
       </c>
-      <c r="E9" s="6">
+      <c r="F16" s="10">
+        <v>5</v>
+      </c>
+      <c r="G16" s="10">
+        <v>15</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="D17" s="10">
+        <v>60</v>
+      </c>
+      <c r="E17" s="10">
+        <v>120</v>
+      </c>
+      <c r="F17" s="10">
+        <v>20</v>
+      </c>
+      <c r="G17" s="10">
+        <v>10</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="D18" s="10">
+        <v>200</v>
+      </c>
+      <c r="E18" s="10">
+        <v>150</v>
+      </c>
+      <c r="F18" s="10">
+        <v>25</v>
+      </c>
+      <c r="G18" s="10">
+        <v>20</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="B21" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22">
+        <v>11</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D22" s="10">
+        <v>70</v>
+      </c>
+      <c r="E22" s="10">
+        <v>100</v>
+      </c>
+      <c r="F22" s="10">
+        <v>30</v>
+      </c>
+      <c r="G22" s="10">
+        <v>14</v>
+      </c>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23">
+        <v>12</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="F9" s="6">
+      <c r="D23" s="10">
+        <v>60</v>
+      </c>
+      <c r="E23" s="10">
+        <v>80</v>
+      </c>
+      <c r="F23" s="10">
+        <v>5</v>
+      </c>
+      <c r="G23" s="10">
+        <v>8</v>
+      </c>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24">
+        <v>15</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="D24" s="10">
+        <v>70</v>
+      </c>
+      <c r="E24" s="10">
+        <v>70</v>
+      </c>
+      <c r="F24" s="10">
+        <v>25</v>
+      </c>
+      <c r="G24" s="10">
+        <v>16</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25">
+        <v>17</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D25" s="10">
+        <v>80</v>
+      </c>
+      <c r="E25" s="10">
+        <v>100</v>
+      </c>
+      <c r="F25" s="10">
+        <v>5</v>
+      </c>
+      <c r="G25" s="10">
+        <v>12</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26">
+        <v>18</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="D26" s="10">
+        <v>70</v>
+      </c>
+      <c r="E26" s="10">
+        <v>100</v>
+      </c>
+      <c r="F26" s="10">
+        <v>15</v>
+      </c>
+      <c r="G26" s="10">
+        <v>16</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27">
+        <v>20</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="D27" s="10">
+        <v>65</v>
+      </c>
+      <c r="E27" s="10">
+        <v>60</v>
+      </c>
+      <c r="F27" s="10">
+        <v>5</v>
+      </c>
+      <c r="G27" s="10">
+        <v>12</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28">
+        <v>22</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="D28" s="10">
+        <v>60</v>
+      </c>
+      <c r="E28" s="10">
+        <v>80</v>
+      </c>
+      <c r="F28" s="10">
         <v>10</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G28" s="10">
+        <v>12</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29">
+        <v>23</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="D29" s="10">
+        <v>70</v>
+      </c>
+      <c r="E29" s="10">
+        <v>110</v>
+      </c>
+      <c r="F29" s="10">
         <v>15</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C10" t="s">
-        <v>66</v>
-      </c>
-      <c r="D10" s="6">
-        <v>90</v>
-      </c>
-      <c r="E10" s="6">
+      <c r="G29" s="10">
+        <v>14</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30">
+        <v>24</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D30" s="10">
+        <v>75</v>
+      </c>
+      <c r="E30" s="10">
+        <v>80</v>
+      </c>
+      <c r="F30" s="10">
+        <v>25</v>
+      </c>
+      <c r="G30" s="10">
+        <v>15</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31">
+        <v>25</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D31" s="10">
         <v>100</v>
       </c>
-      <c r="F10" s="6">
+      <c r="E31" s="10">
+        <v>400</v>
+      </c>
+      <c r="F31" s="10">
+        <v>10</v>
+      </c>
+      <c r="G31" s="10">
+        <v>8</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32">
+        <v>28</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D32" s="10">
+        <v>80</v>
+      </c>
+      <c r="E32" s="10">
+        <v>70</v>
+      </c>
+      <c r="F32" s="10">
         <v>15</v>
       </c>
-      <c r="G10" s="6">
-        <v>14</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>57</v>
+      <c r="G32" s="10">
+        <v>12</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33">
+        <v>29</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D33" s="10">
+        <v>85</v>
+      </c>
+      <c r="E33" s="10">
+        <v>180</v>
+      </c>
+      <c r="F33" s="10">
+        <v>20</v>
+      </c>
+      <c r="G33" s="10">
+        <v>13</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34">
+        <v>30</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="D34" s="10">
+        <v>60</v>
+      </c>
+      <c r="E34" s="10">
+        <v>70</v>
+      </c>
+      <c r="F34" s="10">
+        <v>20</v>
+      </c>
+      <c r="G34" s="10">
+        <v>13</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="I34" s="7" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add remaining 7 characters and 6 skills from AFBElist.xlsx
Implements the characters that were previously left as "still under
consideration" (boxer, gladiator, priest, carrier, merchant, cleaner,
scholar) now that their skills have defined effects in the sheet:
one-two punch (double independent attack), charge (base-seeking
version of blood-scent), tow (drag one ally along when moving, free
of AP cost), commerce (banks a one-round credit bonus per attack),
scavenging (self AP/HP recovery on nearby kills), and analysis
(halves damage from 射程ボーナスN attackers, floored at 5).

Ambiguous mechanics (one-two punch, commerce, tow, analysis) were
confirmed with the user before implementing; charge and scavenging
were unambiguous from the sheet text.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AFBElist.xlsx
+++ b/AFBElist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\遊ぶところ\ゲーム制作\Auto_Formation_Battle_Encounter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B6245A3-50AD-4B70-81DA-3BAF1B8455BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF5EC2F2-34A7-4B01-9BB3-2FD80FCCA05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1B17E940-1388-48E2-89F6-95B4CC23EF03}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="189">
   <si>
     <t>スキル名称</t>
     <rPh sb="3" eb="5">
@@ -540,9 +540,6 @@
     <t>低機動。防衛線・通路封鎖</t>
   </si>
   <si>
-    <t>全体回復20、射程ボーナス1</t>
-  </si>
-  <si>
     <t>範囲2の回復オーラ</t>
   </si>
   <si>
@@ -708,9 +705,6 @@
     <t>僧侶</t>
   </si>
   <si>
-    <t>半径2の回復＋毒解除。首が長い＝範囲広い</t>
-  </si>
-  <si>
     <t>ウマ</t>
   </si>
   <si>
@@ -741,9 +735,6 @@
     <t>解析、射程ボーナス1</t>
   </si>
   <si>
-    <t>敵の防御を崩すデバフオーラ</t>
-  </si>
-  <si>
     <t>ウシ</t>
   </si>
   <si>
@@ -774,9 +765,6 @@
     <t>ボクサー</t>
   </si>
   <si>
-    <t>ワンツー</t>
-  </si>
-  <si>
     <t>1回の攻撃行動で2発。手数の格闘家</t>
   </si>
   <si>
@@ -829,9 +817,6 @@
   </si>
   <si>
     <t>クリーナー</t>
-  </si>
-  <si>
-    <t>死肉あさり</t>
   </si>
   <si>
     <t>死体が出るほど元気になる戦場の掃除屋</t>
@@ -979,13 +964,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>まだ検討中</t>
-    <rPh sb="2" eb="5">
-      <t>ケントウチュウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>採用</t>
     <rPh sb="0" eb="2">
       <t>サイヨウ</t>
@@ -994,10 +972,6 @@
   </si>
   <si>
     <t>スカウト</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>行進曲、射程ボーナス1</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -1099,13 +1073,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>追従</t>
-    <rPh sb="0" eb="2">
-      <t>ツイジュウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>身軽、行進曲</t>
     <rPh sb="0" eb="2">
       <t>ミガル</t>
@@ -1119,34 +1086,6 @@
     <t>建設</t>
     <rPh sb="0" eb="2">
       <t>ケンセツ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>通った道に5tick続く壁を作る（ラウンド終了しても壁は残る）</t>
-    <rPh sb="0" eb="1">
-      <t>トオ</t>
-    </rPh>
-    <rPh sb="3" eb="4">
-      <t>ミチ</t>
-    </rPh>
-    <rPh sb="10" eb="11">
-      <t>ツヅ</t>
-    </rPh>
-    <rPh sb="12" eb="13">
-      <t>カベ</t>
-    </rPh>
-    <rPh sb="14" eb="15">
-      <t>ツク</t>
-    </rPh>
-    <rPh sb="21" eb="23">
-      <t>シュウリョウ</t>
-    </rPh>
-    <rPh sb="26" eb="27">
-      <t>カベ</t>
-    </rPh>
-    <rPh sb="28" eb="29">
-      <t>ノコ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -1210,16 +1149,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>早業、移動ボーナス</t>
-    <rPh sb="0" eb="2">
-      <t>ハヤワザ</t>
-    </rPh>
-    <rPh sb="3" eb="5">
-      <t>イドウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>毒、射程ボーナス１、範囲攻撃</t>
     <rPh sb="0" eb="1">
       <t>ドク</t>
@@ -1253,7 +1182,268 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>聖域、射程ボーナス1</t>
+    <t>早業、移動ボーナス1</t>
+    <rPh sb="0" eb="2">
+      <t>ハヤワザ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>イドウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>通った道に10tick続く壁を作る（ラウンド終了しても壁は残る）</t>
+    <rPh sb="0" eb="1">
+      <t>トオ</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>ミチ</t>
+    </rPh>
+    <rPh sb="11" eb="12">
+      <t>ツヅ</t>
+    </rPh>
+    <rPh sb="13" eb="14">
+      <t>カベ</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>ツク</t>
+    </rPh>
+    <rPh sb="22" eb="24">
+      <t>シュウリョウ</t>
+    </rPh>
+    <rPh sb="27" eb="28">
+      <t>カベ</t>
+    </rPh>
+    <rPh sb="29" eb="30">
+      <t>ノコ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ワンツー</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>攻撃時２回通常攻撃を与える</t>
+    <rPh sb="0" eb="3">
+      <t>コウゲキジ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>カイ</t>
+    </rPh>
+    <rPh sb="5" eb="9">
+      <t>ツウジョウコウゲキ</t>
+    </rPh>
+    <rPh sb="10" eb="11">
+      <t>アタ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ワンツー、攻撃消費１</t>
+    <rPh sb="5" eb="9">
+      <t>コウゲキショウヒ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>全体回復20、射程ボーナス1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>全体回復10、射程ボーナス2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>範囲3の回復オーラ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>突進</t>
+    <rPh sb="0" eb="2">
+      <t>トッシン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>指示は聞かず近い相手の拠点に最短で近づく</t>
+    <rPh sb="0" eb="2">
+      <t>シジ</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="6" eb="7">
+      <t>チカ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>アイテ</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>キョテン</t>
+    </rPh>
+    <rPh sb="14" eb="16">
+      <t>サイタン</t>
+    </rPh>
+    <rPh sb="17" eb="18">
+      <t>チカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>牽引</t>
+    <rPh sb="0" eb="2">
+      <t>ケンイン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>移動時、攻撃範囲にいる味方１体を一緒に動かす。</t>
+    <rPh sb="0" eb="2">
+      <t>イドウ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ジ</t>
+    </rPh>
+    <rPh sb="4" eb="8">
+      <t>コウゲキハンイ</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>ミカタ</t>
+    </rPh>
+    <rPh sb="14" eb="15">
+      <t>タイ</t>
+    </rPh>
+    <rPh sb="16" eb="18">
+      <t>イッショ</t>
+    </rPh>
+    <rPh sb="19" eb="20">
+      <t>ウゴ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>行進曲、射程ボーナス1、追従2</t>
+    <rPh sb="12" eb="14">
+      <t>ツイジュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>追従2</t>
+    <rPh sb="0" eb="2">
+      <t>ツイジュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>商売</t>
+    <rPh sb="0" eb="2">
+      <t>ショウバイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>１回攻撃につき、次のラウンドでもらえるクレジットを20ずつ増加させる</t>
+    <rPh sb="1" eb="2">
+      <t>カイ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>コウゲキ</t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t>ツギ</t>
+    </rPh>
+    <rPh sb="29" eb="31">
+      <t>ゾウカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>攻撃範囲内にいる敵が倒れるたび、行動力１回復、HP20回復</t>
+    <rPh sb="0" eb="5">
+      <t>コウゲキハンイナイ</t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t>テキ</t>
+    </rPh>
+    <rPh sb="10" eb="11">
+      <t>タオ</t>
+    </rPh>
+    <rPh sb="16" eb="19">
+      <t>コウドウリョク</t>
+    </rPh>
+    <rPh sb="20" eb="22">
+      <t>カイフク</t>
+    </rPh>
+    <rPh sb="27" eb="29">
+      <t>カイフク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>死肉あさり</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>死肉あさり、射程ボーナス１</t>
+    <rPh sb="6" eb="8">
+      <t>シャテイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>味方の防御支援</t>
+    <rPh sb="0" eb="2">
+      <t>ミカタ</t>
+    </rPh>
+    <rPh sb="3" eb="7">
+      <t>ボウギョシエン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>解析</t>
+    <rPh sb="0" eb="2">
+      <t>カイセキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自分の攻撃範囲内にいる味方キャラが、射程ボーナスNを持っている敵キャラの攻撃を受ける被ダメージを半減させる。（５以下にはならない）</t>
+    <rPh sb="0" eb="2">
+      <t>ジブン</t>
+    </rPh>
+    <rPh sb="3" eb="8">
+      <t>コウゲキハンイナイ</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>ミカタ</t>
+    </rPh>
+    <rPh sb="18" eb="20">
+      <t>シャテイ</t>
+    </rPh>
+    <rPh sb="26" eb="27">
+      <t>モ</t>
+    </rPh>
+    <rPh sb="31" eb="32">
+      <t>テキ</t>
+    </rPh>
+    <rPh sb="36" eb="38">
+      <t>コウゲキ</t>
+    </rPh>
+    <rPh sb="39" eb="40">
+      <t>ウ</t>
+    </rPh>
+    <rPh sb="42" eb="43">
+      <t>ヒ</t>
+    </rPh>
+    <rPh sb="48" eb="50">
+      <t>ハンゲン</t>
+    </rPh>
+    <rPh sb="56" eb="58">
+      <t>イカ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1699,7 +1889,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19769DCE-A1D1-47E3-BFED-8EA4734B55A4}">
-  <dimension ref="B2:D30"/>
+  <dimension ref="B2:D35"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="9" style="4"/>
@@ -1812,7 +2002,7 @@
         <v>19</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="37.5">
@@ -1908,10 +2098,10 @@
         <v>18</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="37.5">
@@ -1919,10 +2109,10 @@
         <v>19</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="2:4">
@@ -1930,10 +2120,10 @@
         <v>20</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="37.5">
@@ -1941,10 +2131,10 @@
         <v>21</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24" spans="2:4">
@@ -1952,10 +2142,10 @@
         <v>22</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="37.5">
@@ -1963,10 +2153,10 @@
         <v>23</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
     </row>
     <row r="26" spans="2:4">
@@ -1977,18 +2167,18 @@
         <v>32</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="27" spans="2:4">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" ht="37.5">
       <c r="B27" s="3">
         <v>25</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" spans="2:4">
@@ -1996,25 +2186,88 @@
         <v>26</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="29" spans="2:4">
       <c r="B29" s="3">
         <v>27</v>
       </c>
-      <c r="C29" s="1"/>
-      <c r="D29" s="2"/>
+      <c r="C29" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="30" spans="2:4">
       <c r="B30" s="3">
         <v>28</v>
       </c>
-      <c r="C30" s="1"/>
-      <c r="D30" s="2"/>
+      <c r="C30" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4">
+      <c r="B31" s="3">
+        <v>29</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4" ht="37.5">
+      <c r="B32" s="3">
+        <v>30</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4">
+      <c r="B33" s="3">
+        <v>31</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" ht="56.25">
+      <c r="B34" s="3">
+        <v>32</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4">
+      <c r="B35" s="3">
+        <v>33</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>176</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -2024,7 +2277,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14515E83-A93E-48F7-8531-5F98695B0245}">
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="16.125" customWidth="1"/>
@@ -2035,10 +2288,10 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="B1" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>35</v>
@@ -2064,10 +2317,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D2" s="6">
         <v>50</v>
@@ -2093,10 +2346,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D3" s="6">
         <v>60</v>
@@ -2122,10 +2375,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D4" s="6">
         <v>65</v>
@@ -2151,10 +2404,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D5" s="6">
         <v>60</v>
@@ -2169,7 +2422,7 @@
         <v>12</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>47</v>
@@ -2180,10 +2433,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D6" s="6">
         <v>70</v>
@@ -2198,10 +2451,10 @@
         <v>10</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2209,10 +2462,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D7" s="6">
         <v>75</v>
@@ -2227,10 +2480,10 @@
         <v>10</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2238,10 +2491,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D8" s="6">
         <v>70</v>
@@ -2256,10 +2509,10 @@
         <v>15</v>
       </c>
       <c r="H8" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2267,10 +2520,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D9" s="6">
         <v>90</v>
@@ -2285,10 +2538,10 @@
         <v>14</v>
       </c>
       <c r="H9" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="I9" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2296,10 +2549,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" t="s">
         <v>69</v>
-      </c>
-      <c r="C10" t="s">
-        <v>70</v>
       </c>
       <c r="D10" s="6">
         <v>45</v>
@@ -2325,10 +2578,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>75</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>76</v>
       </c>
       <c r="D11" s="9">
         <v>65</v>
@@ -2343,10 +2596,10 @@
         <v>13</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -2354,10 +2607,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D12" s="9">
         <v>30</v>
@@ -2375,7 +2628,7 @@
         <v>41</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -2383,10 +2636,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D13" s="9">
         <v>75</v>
@@ -2401,10 +2654,10 @@
         <v>10</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -2412,10 +2665,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>88</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>89</v>
       </c>
       <c r="D14" s="9">
         <v>110</v>
@@ -2430,10 +2683,10 @@
         <v>15</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -2441,10 +2694,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>83</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>84</v>
       </c>
       <c r="D15" s="9">
         <v>75</v>
@@ -2459,10 +2712,10 @@
         <v>14</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -2470,10 +2723,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D16" s="9">
         <v>80</v>
@@ -2488,10 +2741,10 @@
         <v>15</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>152</v>
+        <v>179</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -2499,10 +2752,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="D17" s="9">
         <v>60</v>
@@ -2517,10 +2770,10 @@
         <v>10</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -2528,10 +2781,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>81</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>82</v>
       </c>
       <c r="D18" s="9">
         <v>200</v>
@@ -2549,7 +2802,7 @@
         <v>9</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -2557,10 +2810,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D19" s="9">
         <v>100</v>
@@ -2575,10 +2828,10 @@
         <v>8</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -2586,10 +2839,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D20" s="9">
         <v>75</v>
@@ -2604,10 +2857,10 @@
         <v>15</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -2615,10 +2868,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" s="9" t="s">
         <v>77</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>78</v>
       </c>
       <c r="D21" s="9">
         <v>70</v>
@@ -2633,10 +2886,10 @@
         <v>14</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -2644,10 +2897,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D22" s="9">
         <v>80</v>
@@ -2662,10 +2915,10 @@
         <v>12</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="18" customHeight="1">
@@ -2673,10 +2926,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C23" s="9" t="s">
         <v>79</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>80</v>
       </c>
       <c r="D23" s="9">
         <v>60</v>
@@ -2691,10 +2944,10 @@
         <v>8</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -2702,10 +2955,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C24" s="9" t="s">
         <v>86</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>87</v>
       </c>
       <c r="D24" s="9">
         <v>80</v>
@@ -2717,75 +2970,111 @@
         <v>25</v>
       </c>
       <c r="G24" s="9">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="D25" s="9">
+        <v>70</v>
+      </c>
+      <c r="E25" s="9">
+        <v>110</v>
+      </c>
+      <c r="F25" s="9">
+        <v>15</v>
+      </c>
+      <c r="G25" s="9">
+        <v>14</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="D26" s="9">
+        <v>85</v>
+      </c>
+      <c r="E26" s="9">
+        <v>180</v>
+      </c>
+      <c r="F26" s="9">
+        <v>25</v>
+      </c>
+      <c r="G26" s="9">
+        <v>13</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="C25" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="D25" s="9">
-        <v>80</v>
-      </c>
-      <c r="E25" s="9">
+      <c r="D27" s="9">
         <v>100</v>
       </c>
-      <c r="F25" s="9">
+      <c r="E27" s="9">
+        <v>100</v>
+      </c>
+      <c r="F27" s="9">
         <v>5</v>
       </c>
-      <c r="G25" s="9">
+      <c r="G27" s="9">
         <v>12</v>
       </c>
-      <c r="H25" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-    </row>
-    <row r="27" spans="1:9">
-      <c r="B27" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
+      <c r="H27" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="28" spans="1:9">
       <c r="A28">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D28" s="9">
         <v>70</v>
@@ -2800,21 +3089,21 @@
         <v>16</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D29" s="9">
         <v>65</v>
@@ -2823,132 +3112,74 @@
         <v>60</v>
       </c>
       <c r="F29" s="9">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G29" s="9">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="D30" s="9">
         <v>60</v>
       </c>
       <c r="E30" s="9">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="F30" s="9">
         <v>10</v>
       </c>
       <c r="G30" s="9">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>111</v>
+        <v>185</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="D31" s="9">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E31" s="9">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="F31" s="9">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="G31" s="9">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9">
-      <c r="A32">
-        <v>29</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="C32" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="D32" s="9">
-        <v>85</v>
-      </c>
-      <c r="E32" s="9">
-        <v>180</v>
-      </c>
-      <c r="F32" s="9">
-        <v>20</v>
-      </c>
-      <c r="G32" s="9">
-        <v>13</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="I32" s="7" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9">
-      <c r="A33">
-        <v>30</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="D33" s="9">
-        <v>60</v>
-      </c>
-      <c r="E33" s="9">
-        <v>70</v>
-      </c>
-      <c r="F33" s="9">
-        <v>20</v>
-      </c>
-      <c r="G33" s="9">
-        <v>13</v>
-      </c>
-      <c r="H33" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="I33" s="7" t="s">
-        <v>135</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>